<commit_message>
Answer-quality evaluation with verification pass
</commit_message>
<xml_diff>
--- a/evaluation/answers/20260925-231936/grading.xlsx
+++ b/evaluation/answers/20260925-231936/grading.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\suman\Downloads\RAG_Project_JU\rag-backend\evaluation\answers\20260925-231936\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{82C5EE64-607A-4DF1-AD55-40AA4A610BA6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F972DFE6-D03C-4B69-84CF-90634ED3BFF6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="663" uniqueCount="382">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="663" uniqueCount="386">
   <si>
     <t>Docwise — answer quality grading</t>
   </si>
@@ -3756,6 +3756,18 @@
   </si>
   <si>
     <t>The answer was not in the context, the model just hallucinates it or he adds it up.</t>
+  </si>
+  <si>
+    <t>তথ্যটি context-এ বাংলায় ছিল, মডেল অনুবাদ করেছে</t>
+  </si>
+  <si>
+    <t>partial</t>
+  </si>
+  <si>
+    <t>মূল যুক্তি context-এ আছে, বিস্তারিত যোগ করা</t>
+  </si>
+  <si>
+    <t>মূল কারণ context-এ স্পষ্ট আছে</t>
   </si>
 </sst>
 </file>
@@ -5827,13 +5839,13 @@
         <v>1</v>
       </c>
       <c r="K34" s="7" t="s">
-        <v>380</v>
+        <v>383</v>
       </c>
       <c r="L34" s="7" t="s">
         <v>379</v>
       </c>
       <c r="M34" s="8" t="s">
-        <v>381</v>
+        <v>384</v>
       </c>
       <c r="N34" s="5" t="s">
         <v>42</v>
@@ -5874,13 +5886,13 @@
         <v>1</v>
       </c>
       <c r="K35" s="7" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="L35" s="7" t="s">
         <v>379</v>
       </c>
       <c r="M35" s="8" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="N35" s="5" t="s">
         <v>66</v>
@@ -5966,13 +5978,13 @@
         <v>1</v>
       </c>
       <c r="K37" s="7" t="s">
-        <v>380</v>
+        <v>383</v>
       </c>
       <c r="L37" s="7" t="s">
         <v>379</v>
       </c>
       <c r="M37" s="8" t="s">
-        <v>381</v>
+        <v>385</v>
       </c>
       <c r="N37" s="5" t="s">
         <v>42</v>

</xml_diff>